<commit_message>
Add bus & room-key outstanding trackers + RoomGroup room workflow
</commit_message>
<xml_diff>
--- a/data/Attendee_List_Template.xlsx
+++ b/data/Attendee_List_Template.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -446,9 +446,10 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="29" customWidth="1" min="7" max="7"/>
     <col width="27" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="37" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,15 +495,20 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>RoomGroup</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Room</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>RoomNote</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -551,17 +557,22 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Hotel room number (pre-assign here if known)</t>
+          <t>房间分组 — same code = same room (e.g. R01). Fill BEFORE camp.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>e.g. roommate names, gender block</t>
+          <t>LEAVE BLANK — actual room number auto-filled at check-in (3pm)</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>allergies, dietary, special needs…</t>
+          <t>e.g. gender block, special needs</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>allergies, dietary, etc.</t>
         </is>
       </c>
     </row>
@@ -598,9 +609,14 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>R01</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
@@ -635,9 +651,14 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>R02</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
         <is>
           <t>负责报到 Registration lead</t>
         </is>
@@ -665,7 +686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -726,43 +747,50 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6. Room: pre-assign here if you have planned rooming; the check-in</t>
+          <t>6. RoomGroup: give everyone sharing a room the SAME code (e.g. R01).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">   screen will then show the room number when you scan them.</t>
+          <t xml:space="preserve">   Leave Room blank — you type each real room number on the Rooms tab</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   at 3pm, and it auto-fills to every member when you scan them in.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>WHEN DONE: send this file back. The generator will:</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • assign each person an ID + security token</t>
+          <t>WHEN DONE: send this file back. The generator will:</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • print all the name tags (front = name, back = QR code)</t>
+          <t xml:space="preserve">  • assign each person an ID + security token</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • print all the name tags (front = name, back = QR code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t xml:space="preserve">  • produce the import file to paste into the Google Sheet.</t>
         </is>

</xml_diff>

<commit_message>
Per-family room keys, key-return tracker, Leader role
</commit_message>
<xml_diff>
--- a/data/Attendee_List_Template.xlsx
+++ b/data/Attendee_List_Template.xlsx
@@ -442,7 +442,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="29" customWidth="1" min="7" max="7"/>
     <col width="27" customWidth="1" min="8" max="8"/>
@@ -537,7 +537,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Attendee or Organiser</t>
+          <t>Attendee / Organiser / Leader (组长)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -667,7 +667,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="E3:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Attendee,Organiser"</formula1>
+      <formula1>"Attendee,Organiser,Leader"</formula1>
     </dataValidation>
     <dataValidation sqref="G3:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>

</xml_diff>

<commit_message>
Add Arrival + Ice-breaker checkpoints; reserve CampGroup/Emergency; 🔎 Lookup with per-activity status
</commit_message>
<xml_diff>
--- a/data/Attendee_List_Template.xlsx
+++ b/data/Attendee_List_Template.xlsx
@@ -435,21 +435,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="29" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="37" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="8" max="8"/>
+    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="35" customWidth="1" min="11" max="11"/>
+    <col width="37" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,40 +477,50 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>CampGroup</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>BusTo</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>BusBack</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>RoomGroup</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Room</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>RoomNote</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -537,40 +549,50 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>紧急联络人 emergency contact (name + phone)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>Attendee / Organiser / Leader (组长)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>小组 / cell group / family</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>营内分组 (ice-breaker/devotion group) — fill later, can leave blank</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Y if taking the church bus TO the venue, else N</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Y if taking the bus BACK to church, else N</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>房间分组 — same code = same room (e.g. R01). Fill BEFORE camp.</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>LEAVE BLANK — actual room number auto-filled at check-in (3pm)</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>e.g. gender block, special needs</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>allergies, dietary, etc.</t>
         </is>
@@ -591,32 +613,38 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>母亲 Mum 0111</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Attendee</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>青年组 Youth</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>R01</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
@@ -633,32 +661,38 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>配偶 Spouse 0122</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Organiser</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>后勤 Logistics</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>R02</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
         <is>
           <t>负责报到 Registration lead</t>
         </is>
@@ -666,13 +700,13 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="E3:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F3:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Attendee,Organiser,Leader"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I3:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J3:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Merge to single Group; by-Group + arrival dashboards; group filter in lookup; hide roles; clearer errors
</commit_message>
<xml_diff>
--- a/data/Attendee_List_Template.xlsx
+++ b/data/Attendee_List_Template.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -443,15 +443,14 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="37" customWidth="1" min="8" max="8"/>
-    <col width="29" customWidth="1" min="9" max="9"/>
-    <col width="27" customWidth="1" min="10" max="10"/>
-    <col width="35" customWidth="1" min="11" max="11"/>
-    <col width="37" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="37" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="37" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,35 +491,30 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>CampGroup</t>
+          <t>BusTo</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>BusTo</t>
+          <t>BusBack</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>BusBack</t>
+          <t>RoomGroup</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>RoomGroup</t>
+          <t>Room</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Room</t>
+          <t>RoomNote</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>RoomNote</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -554,45 +548,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Attendee / Organiser / Leader (组长)</t>
+          <t>Attendee / Organiser / Leader (used for counts; not displayed)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>小组 / cell group / family</t>
+          <t>组别 / 营内分组 — the camp activity group (follows them to 灵修 etc.)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>营内分组 (ice-breaker/devotion group) — fill later, can leave blank</t>
+          <t>Y if taking the church bus TO the venue, else N</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Y if taking the church bus TO the venue, else N</t>
+          <t>Y if taking the bus BACK to church, else N</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Y if taking the bus BACK to church, else N</t>
+          <t>房间分组 — same code = same room (e.g. R01). Fill BEFORE camp.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>房间分组 — same code = same room (e.g. R01). Fill BEFORE camp.</t>
+          <t>LEAVE BLANK — actual room number auto-filled at check-in (3pm)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>LEAVE BLANK — actual room number auto-filled at check-in (3pm)</t>
+          <t>e.g. gender block, special needs</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>e.g. gender block, special needs</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>allergies, dietary, etc.</t>
         </is>
@@ -623,10 +612,14 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>青年组 Youth</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>A 组</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>Y</t>
@@ -634,17 +627,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
           <t>R01</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
@@ -671,10 +659,14 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>后勤 Logistics</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>B 组</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>N</t>
@@ -682,19 +674,14 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
           <t>R02</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>负责报到 Registration lead</t>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>负责报到</t>
         </is>
       </c>
     </row>
@@ -703,10 +690,10 @@
     <dataValidation sqref="F3:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Attendee,Organiser,Leader"</formula1>
     </dataValidation>
-    <dataValidation sqref="I3:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="J3:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I3:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>